<commit_message>
Deploy HydroGeo Field Survey & Unified Excel Hub with Save & Dedup engine and offline cadastral micro-packs
</commit_message>
<xml_diff>
--- a/Integrated_Master_Template.xlsx
+++ b/Integrated_Master_Template.xlsx
@@ -5704,7 +5704,7 @@
     <col width="4.1796875" customWidth="1" style="120" min="6" max="6"/>
     <col width="13.54296875" customWidth="1" style="120" min="7" max="7"/>
     <col width="5.81640625" customWidth="1" style="120" min="8" max="8"/>
-    <col width="4.7265625" customWidth="1" style="120" min="9" max="9"/>
+    <col width="5.5" customWidth="1" style="120" min="9" max="9"/>
     <col width="6" customWidth="1" style="120" min="10" max="11"/>
     <col width="13.453125" customWidth="1" style="120" min="12" max="12"/>
     <col width="6.453125" customWidth="1" style="120" min="13" max="13"/>
@@ -10555,7 +10555,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AM2"/>
+  <dimension ref="A1:Y1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <sheetData>
     <row r="1" ht="28" customHeight="1" s="120">
@@ -10685,7 +10685,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>